<commit_message>
Updated Literature Matrix File
</commit_message>
<xml_diff>
--- a/Papers/Literature Matrix.xlsx
+++ b/Papers/Literature Matrix.xlsx
@@ -1,20 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\deep-doc-clustering\Papers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86BB82E3-39BC-4117-9112-91FE02CDD979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55EF8BAD-FC7E-4323-956A-53DFD5C8E726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="831" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Literature Matrix" sheetId="1" r:id="rId1"/>
+    <sheet name="Keywords" sheetId="3" r:id="rId2"/>
+    <sheet name="Terms Dictionary" sheetId="8" r:id="rId3"/>
+    <sheet name="Representational Modules" sheetId="2" r:id="rId4"/>
+    <sheet name="Clustering Modules" sheetId="9" r:id="rId5"/>
+    <sheet name="Datasets" sheetId="5" r:id="rId6"/>
+    <sheet name="Repositories" sheetId="6" r:id="rId7"/>
+    <sheet name="Eval Metrics" sheetId="7" r:id="rId8"/>
+    <sheet name="Potential Gaps" sheetId="11" r:id="rId9"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Terms Dictionary'!$A$1:$B$9</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="101">
   <si>
     <t>Year</t>
   </si>
@@ -78,14 +89,271 @@
     <t>Captured long term semantics (Inter Document Semantics) via Transformer-GCN Fusion (SOTA)</t>
   </si>
   <si>
-    <t>Citation Structure</t>
+    <t>Keywords</t>
+  </si>
+  <si>
+    <t>Deep Clustering</t>
+  </si>
+  <si>
+    <t>Unsupervised Learning</t>
+  </si>
+  <si>
+    <t>Representational Learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Document Clustering </t>
+  </si>
+  <si>
+    <t>Dicrimintative Representation</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
+    <t>Shallow Clustering</t>
+  </si>
+  <si>
+    <t>The shallow (non-deep) clustering takes the feature vectors of the instances as input and outputs the clustering result without deep neural networks.</t>
+  </si>
+  <si>
+    <t>The deep clustering aims to cluster unstructured data or high-dimensional data with deep neural networks</t>
+  </si>
+  <si>
+    <t>Hard Clustering</t>
+  </si>
+  <si>
+    <t>Soft Clustering</t>
+  </si>
+  <si>
+    <t>The output of hard clustering is a discrete one-hot cluster label yi for each instance xi</t>
+  </si>
+  <si>
+    <t>The output of soft clustering is a continuous cluster assignment probabilistic vector zi</t>
+  </si>
+  <si>
+    <t>Partitioning Clustering</t>
+  </si>
+  <si>
+    <t>Overlapping Clustering</t>
+  </si>
+  <si>
+    <t>Making K partitions of datasets using hard clustering</t>
+  </si>
+  <si>
+    <t>A dataset can be part of multiple clusters</t>
+  </si>
+  <si>
+    <t>Representational Learning Modules</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Auto-Encoder</t>
+  </si>
+  <si>
+    <t>Can be used as representational learning module that learn compact, informative latent features by reconstructing the input through a constrained bottleneck, forcing the model to preserve structure while discarding noise.</t>
+  </si>
+  <si>
+    <t>Weakness</t>
+  </si>
+  <si>
+    <t>Deep Generative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deep generative representation learning uses models like VAEs and GANs to learn latent representations by modeling the data distribution, enabling flexible, interpretable, and generative embeddings.
+</t>
+  </si>
+  <si>
+    <t>Struggle to effectively incorporate clustering information during training, often relying on weak distributional assumptions (e.g., Gaussian mixtures) that fail for complex data.</t>
+  </si>
+  <si>
+    <t>Learns representations on an individual instance
+basis, often overlooking the interconnections between different instances. Consequently, in the
+embedding space, instances may not be distinctly separated, leading to suboptimal clustering
+results.</t>
+  </si>
+  <si>
+    <t>Mutual Information Maximization</t>
+  </si>
+  <si>
+    <t>Focus on instance level similarity, so they often fail to explicitly model cluster semantic structure across different data instances.</t>
+  </si>
+  <si>
+    <t>Contrastive</t>
+  </si>
+  <si>
+    <t>Contrastive learning is one of the most popular unsupervised representation learning techniques
+in recent years. The basic idea is to pull a positive pair of instances close while pushing a negative
+pair of instances far away, which is also known as instance discrimination.</t>
+  </si>
+  <si>
+    <t>Relies heavily on quality positive/negative pairs and large batch sizes, and if negatives are poorly chosen, it can distort cluster structure or cause representation collapse.</t>
+  </si>
+  <si>
+    <t>Clustering Friendly</t>
+  </si>
+  <si>
+    <t>Explicitly optimizes embeddings to match specific clustering objectives e.g., K-means centroids or spectral orthogonality, directly improving clustering performance.</t>
+  </si>
+  <si>
+    <t>Method Specific, limiting generalization</t>
+  </si>
+  <si>
+    <t>Subspace</t>
+  </si>
+  <si>
+    <t>Maps data into low dimensional subspaces using the self-expressiveness assumption, where each instance is represented as a combination of others from the same subspace.</t>
+  </si>
+  <si>
+    <t>Computationally expensive and difficult to scale, especially for large datasets where subspace selection and assignment become complex.</t>
+  </si>
+  <si>
+    <t>Data Type Specific</t>
+  </si>
+  <si>
+    <t>Tailors architectures to images, text, videos, and graphs e.g., CNNs/ViTs, language models, spatiotemporal networks, GNNs to extract more suitable features for deep clustering.</t>
+  </si>
+  <si>
+    <t>Mutual information maximization learns embeddings by enforcing high dependence between different views of the same data instances e.g., sentence–context, augmented sentences, or layer-wise representations, ensuring semantic consistency.</t>
+  </si>
+  <si>
+    <t>Clustering Modules</t>
+  </si>
+  <si>
+    <t>Relation Matching</t>
+  </si>
+  <si>
+    <t>links representation learning and clustering by aligning instance to cluster (I2C) and instance to instance (I2I) relationships in the embedding space. Use cosine similarity or euclidean distance.</t>
+  </si>
+  <si>
+    <t>Computationally expensive and sensitive to noisy relations</t>
+  </si>
+  <si>
+    <t>Pseudo labeling applies semi-supervised learning to deep clustering by generating confident pseudo labels and using them either to supervise individual instances or to enforce must-link / cannot-link relations in embedding space.</t>
+  </si>
+  <si>
+    <t>Its performance is highly sensitive to pseudo-label quality, which depends on model initialization and hyperparameters, making it unstable in fully unsupervised settings.</t>
+  </si>
+  <si>
+    <t>Pseudo Labeling</t>
+  </si>
+  <si>
+    <t>Self-Training</t>
+  </si>
+  <si>
+    <t>KL Divergence</t>
+  </si>
+  <si>
+    <t>KL-divergence is commonly used in soft clustering to measure how different the predicted probability distribution is from a target or reference distribution.</t>
+  </si>
+  <si>
+    <t>Self-training deep clustering refines cluster assignments by minimizing KL-divergence between predicted soft assignments and a sharpened auxiliary distribution, encouraging confident, near one-hot clustering.</t>
+  </si>
+  <si>
+    <t>It is sensitive to class imbalance and early incorrect assignments.</t>
+  </si>
+  <si>
+    <t>Student's t-distribution</t>
+  </si>
+  <si>
+    <t>Student’s t-distribution is a probability distribution similar to a Gaussian but with heavier tails, meaning it assigns higher probability to values far from the mean.</t>
+  </si>
+  <si>
+    <t>Data dependent, requiring different models and design choices per modality</t>
+  </si>
+  <si>
+    <t>Contrastive deep clustering improves clustering by defining positives and negatives at the instance–instance, cluster–cluster, or instance–cluster level, using contrastive loss to make embeddings and clusters more discriminative and robust via data augmentation.</t>
+  </si>
+  <si>
+    <t>Its effectiveness depends on reliable cluster assignments/centroids and augmentations, which can be unstable in early training stages.</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>https://archive.ics.uci.edu/ml/datasets/Reuters-21578+Text+Categorization+Collection</t>
+  </si>
+  <si>
+    <t>Reuters-21578</t>
+  </si>
+  <si>
+    <t>20 Newsgroups</t>
+  </si>
+  <si>
+    <t>http://qwone.com/%7Ejason/20Newsgroups/</t>
+  </si>
+  <si>
+    <t>DOC 50</t>
+  </si>
+  <si>
+    <t>IMDB</t>
+  </si>
+  <si>
+    <t>stackOverflow</t>
+  </si>
+  <si>
+    <t>Others</t>
+  </si>
+  <si>
+    <t>https://github.com/niderhoff/nlp-datasets</t>
+  </si>
+  <si>
+    <t>Metrics</t>
+  </si>
+  <si>
+    <t>Accuracy(ACC)</t>
+  </si>
+  <si>
+    <t>Normalized Mutual
+Information (NMI)</t>
+  </si>
+  <si>
+    <t>Adjusted Rand Index (ARI)</t>
+  </si>
+  <si>
+    <t>Measures the best one-to-one match between predicted clusters and true labels, counting how many instances are correctly assigned after optimal label permutation.</t>
+  </si>
+  <si>
+    <t>NMI quantifies the mutual information between the predicted
+labels and ground truth labels into [0, 1]</t>
+  </si>
+  <si>
+    <t>Measures similarity between predicted and true clusterings by counting pairwise agreements, adjusted for chance (-1 = worst than random, 0 ≈ random, 1 = perfect).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-trained Models haven't been explored a lot for clustering </t>
+  </si>
+  <si>
+    <t>Instances may belong to multiple clusters (overlapping) through unsupervised learning</t>
+  </si>
+  <si>
+    <t>Gaps</t>
+  </si>
+  <si>
+    <t>S.No.</t>
+  </si>
+  <si>
+    <t>How to boost representational learning through clustering remains to be studied</t>
+  </si>
+  <si>
+    <t>leveraging clustering results to extract knowledge and reduce distribution shift in unsupervised transfer learning.</t>
+  </si>
+  <si>
+    <t>contrastive deep clustering</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -93,8 +361,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -107,8 +399,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -116,11 +426,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -131,18 +460,257 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
+  <dxfs count="34">
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -182,6 +750,12 @@
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -203,22 +777,236 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>551506</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4FC3E8E1-B6C0-23B2-A7DA-F39ACCA77D23}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3406140" y="91440"/>
+          <a:ext cx="5938846" cy="3741420"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>6511348</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>91807</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1155420</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>14311</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B120B91A-5568-08F4-1CF6-851CA87BF9BF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6511348" y="8552635"/>
+          <a:ext cx="11092762" cy="4704711"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>3596592</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>184451</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>989762</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>140484</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7665B106-7D52-6621-5BDF-9D5A49252090}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3596592" y="4221430"/>
+          <a:ext cx="8053064" cy="3498522"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}" name="Table1" displayName="Table1" ref="A1:J2" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:J2" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}"/>
-  <tableColumns count="10">
-    <tableColumn id="2" xr3:uid="{DB226ECB-CD8C-42E9-A3A4-AF7E80A56DFC}" name="Year" dataDxfId="11"/>
-    <tableColumn id="1" xr3:uid="{F82E7BA8-7A49-4869-B7FE-750ECF9B2D7D}" name="Paper" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{C3BB9434-C5C6-4832-9955-1B33CEEFC6C8}" name="Embedding Method" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{469AE431-C88B-47B2-A8BB-C9262A37B57A}" name="Clustering Strategy" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{192B4256-B842-4B73-8E3F-F63D9AFCDBF9}" name="Evaluation Metrics" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{9E317EA9-476B-4EA5-8E71-3298757B143C}" name="Dataset" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{E5470C89-57EA-4C48-BA16-5695CCD21AA2}" name="Strengths" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{EC789573-2750-4DF9-B276-745D8F66A3A7}" name="Weaknesses" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{93B755E8-002C-46C7-919C-B7D00E5A91B3}" name="Summary" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{0A195EEB-7E51-44CA-A65D-FE0D0113FB60}" name="Citation Structure" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}" name="Table1" displayName="Table1" ref="A1:I2" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+  <autoFilter ref="A1:I2" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}"/>
+  <tableColumns count="9">
+    <tableColumn id="2" xr3:uid="{DB226ECB-CD8C-42E9-A3A4-AF7E80A56DFC}" name="Year" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{F82E7BA8-7A49-4869-B7FE-750ECF9B2D7D}" name="Paper" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{C3BB9434-C5C6-4832-9955-1B33CEEFC6C8}" name="Embedding Method" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{469AE431-C88B-47B2-A8BB-C9262A37B57A}" name="Clustering Strategy" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{192B4256-B842-4B73-8E3F-F63D9AFCDBF9}" name="Evaluation Metrics" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{9E317EA9-476B-4EA5-8E71-3298757B143C}" name="Dataset" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{E5470C89-57EA-4C48-BA16-5695CCD21AA2}" name="Strengths" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{EC789573-2750-4DF9-B276-745D8F66A3A7}" name="Weaknesses" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{93B755E8-002C-46C7-919C-B7D00E5A91B3}" name="Summary" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C76C095F-3BC5-4629-8535-0976DE13D2F7}" name="Table6" displayName="Table6" ref="A1:B9" totalsRowShown="0" headerRowDxfId="17" dataDxfId="18">
+  <autoFilter ref="A1:B9" xr:uid="{C02DD467-9E9B-432F-B259-B47BDB2E8030}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{B8BCBE5A-2975-4202-AF24-8D605D4839B0}" name="Term" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{02082F22-E9E9-45E2-BCEE-26DEF17426CD}" name="Explanation" dataDxfId="16"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8078C8ED-6189-4B3C-AE11-C6DEA86A8B3B}" name="Table3" displayName="Table3" ref="A1:C8" totalsRowShown="0" headerRowDxfId="19">
+  <autoFilter ref="A1:C8" xr:uid="{8078C8ED-6189-4B3C-AE11-C6DEA86A8B3B}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{08DD60B6-8716-46D2-95ED-290B15FC56B3}" name="Representational Learning Modules" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{F70ECD39-FBA0-492C-851B-05440433BB6F}" name="Description" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{6E71AC32-9BCA-4E74-8E24-803673D80ECC}" name="Weakness" dataDxfId="20"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{E2D47D74-1281-4F3E-82DB-74C1BAE35332}" name="Table10" displayName="Table10" ref="A1:C5" totalsRowShown="0" headerRowDxfId="6" tableBorderDxfId="10">
+  <autoFilter ref="A1:C5" xr:uid="{E2D47D74-1281-4F3E-82DB-74C1BAE35332}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{906EB2EE-0A52-4F48-B0E5-9DC200CED6D2}" name="Clustering Modules" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{F75ED1A2-4791-4A18-8C67-41229F776CE0}" name="Description" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{D62FA453-7E2C-4BA9-93CA-E77C1D07FA1A}" name="Weakness" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B1B50FA9-8B75-4B36-AFBC-143695D985C1}" name="Table9" displayName="Table9" ref="A1:B7" totalsRowShown="0" headerRowDxfId="11" dataDxfId="12">
+  <autoFilter ref="A1:B7" xr:uid="{B1B50FA9-8B75-4B36-AFBC-143695D985C1}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{3A7CE04A-DE22-4AC6-BBB2-45339F6138F7}" name="Name" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{0B0EF4F7-AE8D-4EA4-8EEC-F7FCB91E3280}" name="Link" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{56ECECE1-8DB5-43B1-B5DB-7EC24D2D1789}" name="Table8" displayName="Table8" ref="A1:B4" totalsRowShown="0" headerRowDxfId="13">
+  <autoFilter ref="A1:B4" xr:uid="{56ECECE1-8DB5-43B1-B5DB-7EC24D2D1789}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{C29FF8BC-C149-46BE-AEA9-55B7AA087AC1}" name="Metrics" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{1DE66F54-F599-4ACB-81BF-D4341ACE4E3F}" name="Description" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0DFE8424-B5C7-42F0-8EF1-5F64350460C4}" name="Table7" displayName="Table7" ref="A1:B5" totalsRowShown="0" headerRowDxfId="14">
+  <autoFilter ref="A1:B5" xr:uid="{0DFE8424-B5C7-42F0-8EF1-5F64350460C4}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{EC828149-D73C-4C0C-826C-0F4AA7C10234}" name="S.No." dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{23275512-232B-445A-8104-2B5AF06D489A}" name="Gaps" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -485,25 +1273,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.77734375" style="2" customWidth="1"/>
     <col min="2" max="2" width="94.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="60.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="75.33203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="47.5546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="39" style="2" customWidth="1"/>
     <col min="6" max="6" width="21.88671875" style="3" customWidth="1"/>
     <col min="7" max="7" width="33.77734375" style="2" customWidth="1"/>
     <col min="8" max="8" width="48.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="86.21875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="41.44140625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="33.109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="20.21875" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="1"/>
+    <col min="9" max="9" width="110.5546875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="33.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="20.21875" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -531,11 +1318,8 @@
       <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>2025</v>
       </c>
@@ -562,6 +1346,510 @@
       </c>
       <c r="I2" s="2" t="s">
         <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4356A6C1-D9F9-4DD3-BFAD-397293D70802}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48.21875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="8.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C02DD467-9E9B-432F-B259-B47BDB2E8030}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="51" style="2" customWidth="1"/>
+    <col min="2" max="2" width="148.77734375" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="5" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{910CAD37-1D0E-4531-BA2F-AF4237A942F4}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="107.109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="132.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="109.109375" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="7" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="128.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EB5F05-CA1F-42C0-ACB9-899D9363EEC8}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="72" style="6" customWidth="1"/>
+    <col min="2" max="2" width="83.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="44.21875" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C07D935-71DB-45A3-94F1-4E5CFB282072}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="41.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="58.88671875" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{FDFFD7D6-063B-42AE-A560-97957C52B81E}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{B3829EE8-05F8-4ADA-A260-5F41DC6DAADB}"/>
+    <hyperlink ref="B7" r:id="rId3" xr:uid="{C0A6CBD8-05A5-4716-8C5A-669A3ABD7C6B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId4"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6A4EEFD-FE3B-47CC-B4BD-4F65D457868F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A71D65FD-778C-4AB0-A9FD-4C48D8262705}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="66" style="1" customWidth="1"/>
+    <col min="2" max="2" width="71.5546875" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14A211C0-E1C6-436A-8986-25A43AA682B9}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="108.77734375" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>